<commit_message>
vx_profile: add y_extent_mode=slice_auto and use effective y0/H to avoid empty bins
</commit_message>
<xml_diff>
--- a/out/pipe_flow_2d.xlsx
+++ b/out/pipe_flow_2d.xlsx
@@ -22523,14 +22523,14 @@
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="23" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="23" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -22598,31 +22598,31 @@
         <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>0.08</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>-0.1247118209772335</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>0.138109985980034</v>
       </c>
       <c r="F2" t="n">
-        <v>0.01987121889294599</v>
+        <v>0.09238929787608308</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.02648809986162726</v>
+        <v>0.02399592607330669</v>
       </c>
       <c r="H2" t="n">
-        <v>0.06937833851200335</v>
+        <v>0.02411901666739928</v>
       </c>
       <c r="I2" t="n">
-        <v>0.01987121889294385</v>
+        <v>0.09238929787608337</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>0.1381099859800076</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>-0.1247118209772079</v>
       </c>
     </row>
     <row r="3">
@@ -22633,31 +22633,31 @@
         <v>8</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>0.08</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>0.0639079175248759</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>-0.2062558423414495</v>
       </c>
       <c r="F3" t="n">
-        <v>0.03980038359740282</v>
+        <v>0.1727132686548163</v>
       </c>
       <c r="G3" t="n">
-        <v>0.04253541604137017</v>
+        <v>-0.1163150394825717</v>
       </c>
       <c r="H3" t="n">
-        <v>0.04561115964230899</v>
+        <v>0.1632147403189713</v>
       </c>
       <c r="I3" t="n">
-        <v>0.03980038359738113</v>
+        <v>0.1727132686548645</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>-0.2062558423414629</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>0.06390791752489389</v>
       </c>
     </row>
     <row r="4">
@@ -22668,31 +22668,31 @@
         <v>8</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>0.08</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>0.06166831435293191</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>0.1053466223297573</v>
       </c>
       <c r="F4" t="n">
-        <v>0.05557017816787024</v>
+        <v>0.01212038163911929</v>
       </c>
       <c r="G4" t="n">
-        <v>0.1011432817702251</v>
+        <v>0.04958242098092584</v>
       </c>
       <c r="H4" t="n">
-        <v>0.03116799529728332</v>
+        <v>0.05082576293647788</v>
       </c>
       <c r="I4" t="n">
-        <v>0.05557017816787451</v>
+        <v>0.01212038163924618</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>0.1053466223299266</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>0.06166831435296029</v>
       </c>
     </row>
     <row r="5">
@@ -22703,31 +22703,31 @@
         <v>8</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>0.08</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>0.1055746974575788</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>0.1907454957413182</v>
       </c>
       <c r="F5" t="n">
-        <v>0.04536676564550808</v>
+        <v>-0.00833364735584601</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1097079534289944</v>
+        <v>-0.002912682824081761</v>
       </c>
       <c r="H5" t="n">
-        <v>0.09838747818608863</v>
+        <v>0.1000901410575458</v>
       </c>
       <c r="I5" t="n">
-        <v>0.04536676564585513</v>
+        <v>-0.0083336473559495</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>0.1907454957412621</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>0.1055746974576544</v>
       </c>
     </row>
     <row r="6">
@@ -22738,31 +22738,31 @@
         <v>8</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>0.08</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>0.1376019486762566</v>
       </c>
       <c r="E6" t="n">
-        <v>0.2307763784868531</v>
+        <v>0.03159276438582559</v>
       </c>
       <c r="F6" t="n">
-        <v>0.05125237213062937</v>
+        <v>0.04914462591619033</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1117924725832012</v>
+        <v>0.1013983568999323</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1328432956710083</v>
+        <v>0.1363259129682819</v>
       </c>
       <c r="I6" t="n">
-        <v>0.05125237213034724</v>
+        <v>0.04914462591606659</v>
       </c>
       <c r="J6" t="n">
-        <v>0.2307763784797953</v>
+        <v>0.0315927643850893</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>0.1376019486766278</v>
       </c>
     </row>
     <row r="7">
@@ -22773,31 +22773,31 @@
         <v>8</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>0.08</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>0.08976657872199861</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.0271593363587694</v>
+        <v>0.06596983041621629</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1105136358767233</v>
+        <v>0.1258525233628786</v>
       </c>
       <c r="G7" t="n">
-        <v>0.1088250274347321</v>
+        <v>0.1566449361719087</v>
       </c>
       <c r="H7" t="n">
-        <v>0.1263066900679598</v>
+        <v>0.04447506467620148</v>
       </c>
       <c r="I7" t="n">
-        <v>0.1105136358769074</v>
+        <v>0.1258525233635752</v>
       </c>
       <c r="J7" t="n">
-        <v>-0.02715933635960643</v>
+        <v>0.06596983041585987</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>0.08976657872176577</v>
       </c>
     </row>
     <row r="8">
@@ -22808,31 +22808,31 @@
         <v>8</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>0.08</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>0.03818518547349324</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.02340567582666334</v>
+        <v>0.09726710531833907</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1326014208739966</v>
+        <v>0.08474863855844721</v>
       </c>
       <c r="G8" t="n">
-        <v>0.1278702161160887</v>
+        <v>0.06795063489716949</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1280590002907128</v>
+        <v>0.05962476849817593</v>
       </c>
       <c r="I8" t="n">
-        <v>0.1326014208741591</v>
+        <v>0.08474863855812147</v>
       </c>
       <c r="J8" t="n">
-        <v>-0.02340567582874945</v>
+        <v>0.09726710531813527</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>0.03818518547221279</v>
       </c>
     </row>
     <row r="9">
@@ -22843,31 +22843,31 @@
         <v>8</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>0.08</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>0.07049141667584431</v>
       </c>
       <c r="E9" t="n">
-        <v>0.00590632338030145</v>
+        <v>0.1068052828536393</v>
       </c>
       <c r="F9" t="n">
-        <v>0.1362374648280825</v>
+        <v>0.1536512945659057</v>
       </c>
       <c r="G9" t="n">
-        <v>0.1558004699001167</v>
+        <v>0.1239943501054446</v>
       </c>
       <c r="H9" t="n">
-        <v>0.1516502540986558</v>
+        <v>0.1160632384784225</v>
       </c>
       <c r="I9" t="n">
-        <v>0.136237464827885</v>
+        <v>0.1536512945665001</v>
       </c>
       <c r="J9" t="n">
-        <v>0.005906323382386485</v>
+        <v>0.1068052828535913</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>0.07049141667575597</v>
       </c>
     </row>
     <row r="10">
@@ -22878,31 +22878,31 @@
         <v>8</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>0.08</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>0.1068450819947372</v>
       </c>
       <c r="E10" t="n">
-        <v>0.02058880460745074</v>
+        <v>0.1273831179018263</v>
       </c>
       <c r="F10" t="n">
-        <v>0.1494689365939243</v>
+        <v>0.1484675833352412</v>
       </c>
       <c r="G10" t="n">
-        <v>0.1657384395626071</v>
+        <v>0.1296432096742648</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1711130569415115</v>
+        <v>0.1276809833392841</v>
       </c>
       <c r="I10" t="n">
-        <v>0.1494689365942986</v>
+        <v>0.1484675833350116</v>
       </c>
       <c r="J10" t="n">
-        <v>0.02058880460392718</v>
+        <v>0.1273831179013245</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>0.1068450819942472</v>
       </c>
     </row>
     <row r="11">
@@ -22913,31 +22913,31 @@
         <v>8</v>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>0.08</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>0.1323344828167832</v>
       </c>
       <c r="E11" t="n">
-        <v>0.03030512437201301</v>
+        <v>0.1315542435034637</v>
       </c>
       <c r="F11" t="n">
-        <v>0.1595629609028905</v>
+        <v>0.1450599033592498</v>
       </c>
       <c r="G11" t="n">
-        <v>0.1753052629642945</v>
+        <v>0.1293818513933742</v>
       </c>
       <c r="H11" t="n">
-        <v>0.1923927819647933</v>
+        <v>0.1301119598546073</v>
       </c>
       <c r="I11" t="n">
-        <v>0.1595629609002498</v>
+        <v>0.145059903359225</v>
       </c>
       <c r="J11" t="n">
-        <v>0.03030512438133151</v>
+        <v>0.1315542435030285</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>0.132334482816365</v>
       </c>
     </row>
   </sheetData>
@@ -23050,7 +23050,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1db5da9ce6fd8c2884826a9980e1ff69b54c9a7f</t>
+          <t>fdd0c13165807eb31cf111d88f107df2c758e2f0</t>
         </is>
       </c>
     </row>
@@ -23086,7 +23086,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>{"debug_vx_profile": {"bins": 8, "enable": true, "every": 50}, "type": "wcsph"}</t>
+          <t>{"debug_vx_profile": {"H": 0.2, "axis": 1, "bins": 8, "component": 0, "enable": true, "every": 50, "gx": 1.0, "nu": 0.01, "out_file": "out/pipe_flow_2d/vx_profile_bins.csv", "use_x_slice": true, "x_slice_width": 0.08, "y0": 0.0, "y_extent_mode": "slice_auto"}, "type": "wcsph"}</t>
         </is>
       </c>
     </row>
@@ -23110,7 +23110,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-02-25T13:02:16.507416+00:00</t>
+          <t>2026-03-03T23:22:57.033895+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
vx_profile: add y_extent_mode=walls and rolling avg for stable Poiseuille validation
</commit_message>
<xml_diff>
--- a/out/pipe_flow_2d.xlsx
+++ b/out/pipe_flow_2d.xlsx
@@ -22523,14 +22523,14 @@
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="23" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -22601,28 +22601,28 @@
         <v>0.08</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.1247118209772335</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>0.138109985980034</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0.09238929787608308</v>
+        <v>0.02055452536214109</v>
       </c>
       <c r="G2" t="n">
-        <v>0.02399592607330669</v>
+        <v>0.02054447156519725</v>
       </c>
       <c r="H2" t="n">
-        <v>0.02411901666739928</v>
+        <v>0.02679659001021851</v>
       </c>
       <c r="I2" t="n">
-        <v>0.09238929787608337</v>
+        <v>0.02055452536214755</v>
       </c>
       <c r="J2" t="n">
-        <v>0.1381099859800076</v>
+        <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>-0.1247118209772079</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -22636,28 +22636,28 @@
         <v>0.08</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0639079175248759</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.2062558423414495</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1727132686548163</v>
+        <v>0.03633541437906722</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.1163150394825717</v>
+        <v>-0.01343664377087245</v>
       </c>
       <c r="H3" t="n">
-        <v>0.1632147403189713</v>
+        <v>0.0797399494963288</v>
       </c>
       <c r="I3" t="n">
-        <v>0.1727132686548645</v>
+        <v>0.03633541437907982</v>
       </c>
       <c r="J3" t="n">
-        <v>-0.2062558423414629</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>0.06390791752489389</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -22671,28 +22671,28 @@
         <v>0.08</v>
       </c>
       <c r="D4" t="n">
-        <v>0.06166831435293191</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1053466223297573</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>0.01212038163911929</v>
+        <v>0.06040133667965118</v>
       </c>
       <c r="G4" t="n">
-        <v>0.04958242098092584</v>
+        <v>0.04761349647926585</v>
       </c>
       <c r="H4" t="n">
-        <v>0.05082576293647788</v>
+        <v>0.04890879421902746</v>
       </c>
       <c r="I4" t="n">
-        <v>0.01212038163924618</v>
+        <v>0.06040133667976511</v>
       </c>
       <c r="J4" t="n">
-        <v>0.1053466223299266</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>0.06166831435296029</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -22706,28 +22706,28 @@
         <v>0.08</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1055746974575788</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>0.1907454957413182</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.00833364735584601</v>
+        <v>0.07290750632708617</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.002912682824081761</v>
+        <v>0.09539602911987255</v>
       </c>
       <c r="H5" t="n">
-        <v>0.1000901410575458</v>
+        <v>0.07199237911829656</v>
       </c>
       <c r="I5" t="n">
-        <v>-0.0083336473559495</v>
+        <v>0.07290750632704862</v>
       </c>
       <c r="J5" t="n">
-        <v>0.1907454957412621</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>0.1055746974576544</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -22741,28 +22741,28 @@
         <v>0.08</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1376019486762566</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>0.03159276438582559</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>0.04914462591619033</v>
+        <v>0.1092968363602842</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1013983568999323</v>
+        <v>0.03626272295856409</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1363259129682819</v>
+        <v>0.08346238694456717</v>
       </c>
       <c r="I6" t="n">
-        <v>0.04914462591606659</v>
+        <v>0.1092968363600086</v>
       </c>
       <c r="J6" t="n">
-        <v>0.0315927643850893</v>
+        <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>0.1376019486766278</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -22776,28 +22776,28 @@
         <v>0.08</v>
       </c>
       <c r="D7" t="n">
-        <v>0.08976657872199861</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>0.06596983041621629</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1258525233628786</v>
+        <v>0.08426102619633785</v>
       </c>
       <c r="G7" t="n">
-        <v>0.1566449361719087</v>
+        <v>0.1034649288043911</v>
       </c>
       <c r="H7" t="n">
-        <v>0.04447506467620148</v>
+        <v>0.0926649753232005</v>
       </c>
       <c r="I7" t="n">
-        <v>0.1258525233635752</v>
+        <v>0.08426102619583682</v>
       </c>
       <c r="J7" t="n">
-        <v>0.06596983041585987</v>
+        <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>0.08976657872176577</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -22811,28 +22811,28 @@
         <v>0.08</v>
       </c>
       <c r="D8" t="n">
-        <v>0.03818518547349324</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>0.09726710531833907</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>0.08474863855844721</v>
+        <v>0.06772614539591615</v>
       </c>
       <c r="G8" t="n">
-        <v>0.06795063489716949</v>
+        <v>0.08457009271339487</v>
       </c>
       <c r="H8" t="n">
-        <v>0.05962476849817593</v>
+        <v>0.06387697462011745</v>
       </c>
       <c r="I8" t="n">
-        <v>0.08474863855812147</v>
+        <v>0.06772614539517403</v>
       </c>
       <c r="J8" t="n">
-        <v>0.09726710531813527</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>0.03818518547221279</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -22846,28 +22846,28 @@
         <v>0.08</v>
       </c>
       <c r="D9" t="n">
-        <v>0.07049141667584431</v>
+        <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>0.1068052828536393</v>
+        <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>0.1536512945659057</v>
+        <v>0.08864834976474181</v>
       </c>
       <c r="G9" t="n">
-        <v>0.1239943501054446</v>
+        <v>0.1509284107085812</v>
       </c>
       <c r="H9" t="n">
-        <v>0.1160632384784225</v>
+        <v>0.1213902362207444</v>
       </c>
       <c r="I9" t="n">
-        <v>0.1536512945665001</v>
+        <v>0.08864834976467362</v>
       </c>
       <c r="J9" t="n">
-        <v>0.1068052828535913</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>0.07049141667575597</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -22881,28 +22881,28 @@
         <v>0.08</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1068450819947372</v>
+        <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>0.1273831179018263</v>
+        <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>0.1484675833352412</v>
+        <v>0.1171140999482817</v>
       </c>
       <c r="G10" t="n">
-        <v>0.1296432096742648</v>
+        <v>0.147819592727893</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1276809833392841</v>
+        <v>0.1289860918103911</v>
       </c>
       <c r="I10" t="n">
-        <v>0.1484675833350116</v>
+        <v>0.1171140999477858</v>
       </c>
       <c r="J10" t="n">
-        <v>0.1273831179013245</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>0.1068450819942472</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -22916,28 +22916,28 @@
         <v>0.08</v>
       </c>
       <c r="D11" t="n">
-        <v>0.1323344828167832</v>
+        <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>0.1315542435034637</v>
+        <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>0.1450599033592498</v>
+        <v>0.1319443631601235</v>
       </c>
       <c r="G11" t="n">
-        <v>0.1293818513933742</v>
+        <v>0.1466548888472708</v>
       </c>
       <c r="H11" t="n">
-        <v>0.1301119598546073</v>
+        <v>0.1289494128799741</v>
       </c>
       <c r="I11" t="n">
-        <v>0.145059903359225</v>
+        <v>0.1319443631596967</v>
       </c>
       <c r="J11" t="n">
-        <v>0.1315542435030285</v>
+        <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>0.132334482816365</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -23050,7 +23050,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>fdd0c13165807eb31cf111d88f107df2c758e2f0</t>
+          <t>ea6b1b86d61a56b09fbdb2de58711df35af56be6</t>
         </is>
       </c>
     </row>
@@ -23086,7 +23086,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>{"debug_vx_profile": {"H": 0.2, "axis": 1, "bins": 8, "component": 0, "enable": true, "every": 50, "gx": 1.0, "nu": 0.01, "out_file": "out/pipe_flow_2d/vx_profile_bins.csv", "use_x_slice": true, "x_slice_width": 0.08, "y0": 0.0, "y_extent_mode": "slice_auto"}, "type": "wcsph"}</t>
+          <t>{"debug_vx_profile": {"H": 0.2, "avg_window_steps": 200, "axis": 1, "bins": 8, "component": 0, "enable": true, "every": 50, "gx": 1.0, "nu": 0.01, "out_file": "out/pipe_flow_2d/vx_profile_bins.csv", "use_x_slice": true, "x_slice_width": 0.08, "y0": 0.0, "y_extent_mode": "walls"}, "type": "wcsph"}</t>
         </is>
       </c>
     </row>
@@ -23110,7 +23110,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-03-03T23:22:57.033895+00:00</t>
+          <t>2026-03-03T23:33:12.774170+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
pipe_flow: use wall-based y extent and widen x-slice for full vx bins
</commit_message>
<xml_diff>
--- a/out/pipe_flow_2d.xlsx
+++ b/out/pipe_flow_2d.xlsx
@@ -23050,7 +23050,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ea6b1b86d61a56b09fbdb2de58711df35af56be6</t>
+          <t>d3c013fdaec34538a45a1e609ea5ce9bbdc9bcb0</t>
         </is>
       </c>
     </row>
@@ -23110,7 +23110,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-03-03T23:33:12.774170+00:00</t>
+          <t>2026-03-03T23:38:17.415308+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>